<commit_message>
Add evaluate.py with match metrics and distance distribution plot
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.1742</v>
+        <v>3.1979</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.4759</v>
+        <v>3.4827</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.5686</v>
+        <v>3.5728</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.0205</v>
+        <v>1.0214</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.6073</v>
+        <v>1.6125</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.7188</v>
+        <v>1.7213</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.3966</v>
+        <v>0.4011</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.458</v>
+        <v>0.4633</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.5477</v>
+        <v>0.5512</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.351</v>
+        <v>0.3522</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.188</v>
+        <v>1.1861</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.5359</v>
+        <v>1.5388</v>
       </c>
       <c r="E13" t="n">
         <v>3</v>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.5573</v>
+        <v>0.5581</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -832,16 +832,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>323410</t>
+          <t>085620</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>미래에셋생명</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.5611</v>
+        <v>0.5605</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
@@ -860,16 +860,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>085620</t>
+          <t>323410</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>미래에셋생명</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.5616</v>
+        <v>0.5621</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.3226</v>
+        <v>0.3243</v>
       </c>
       <c r="E17" t="n">
         <v>1</v>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.3261</v>
+        <v>0.3247</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.3762</v>
+        <v>0.3772</v>
       </c>
       <c r="E19" t="n">
         <v>3</v>
@@ -981,7 +981,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.5842000000000001</v>
+        <v>0.5794</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.8379</v>
+        <v>0.8408</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.9248</v>
+        <v>0.9283</v>
       </c>
       <c r="E22" t="n">
         <v>3</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.6541</v>
+        <v>0.6546</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.8374</v>
+        <v>0.8398</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.9918</v>
+        <v>0.9927</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3.0447</v>
+        <v>3.0448</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3.0893</v>
+        <v>3.0895</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.0963</v>
+        <v>3.0965</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.7719</v>
+        <v>0.763</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2.2189</v>
+        <v>2.2241</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2.3624</v>
+        <v>2.3658</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.1554</v>
+        <v>0.1557</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.1671</v>
+        <v>0.1676</v>
       </c>
       <c r="E33" t="n">
         <v>2</v>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.2154</v>
+        <v>0.2162</v>
       </c>
       <c r="E34" t="n">
         <v>3</v>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4.4793</v>
+        <v>4.4797</v>
       </c>
       <c r="E38" t="n">
         <v>1</v>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4.5135</v>
+        <v>4.5137</v>
       </c>
       <c r="E39" t="n">
         <v>2</v>
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1835</v>
+        <v>0.1826</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.2047</v>
+        <v>0.2053</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.3199</v>
+        <v>0.3162</v>
       </c>
       <c r="E43" t="n">
         <v>3</v>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.0958</v>
+        <v>0.09669999999999999</v>
       </c>
       <c r="E44" t="n">
         <v>1</v>
@@ -1672,16 +1672,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>097230</t>
+          <t>010140</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.112</v>
+        <v>0.1121</v>
       </c>
       <c r="E45" t="n">
         <v>2</v>
@@ -1700,16 +1700,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>010140</t>
+          <t>097230</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.1155</v>
+        <v>0.1126</v>
       </c>
       <c r="E46" t="n">
         <v>3</v>
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.2506</v>
+        <v>0.2533</v>
       </c>
       <c r="E48" t="n">
         <v>2</v>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.4228</v>
+        <v>0.4221</v>
       </c>
       <c r="E49" t="n">
         <v>3</v>
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.0193</v>
+        <v>1.0206</v>
       </c>
       <c r="E50" t="n">
         <v>1</v>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1.2088</v>
+        <v>1.2095</v>
       </c>
       <c r="E51" t="n">
         <v>2</v>
@@ -1896,16 +1896,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>068270</t>
+          <t>128940</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.2334</v>
+        <v>0.2325</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
@@ -1924,16 +1924,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>128940</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.2373</v>
+        <v>0.2347</v>
       </c>
       <c r="E54" t="n">
         <v>2</v>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.286</v>
+        <v>0.2847</v>
       </c>
       <c r="E55" t="n">
         <v>3</v>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1.7476</v>
+        <v>1.7475</v>
       </c>
       <c r="E57" t="n">
         <v>2</v>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.7481</v>
+        <v>1.7482</v>
       </c>
       <c r="E58" t="n">
         <v>3</v>
@@ -2101,7 +2101,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.1012</v>
+        <v>0.1025</v>
       </c>
       <c r="E60" t="n">
         <v>2</v>
@@ -2129,7 +2129,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.1086</v>
+        <v>0.1067</v>
       </c>
       <c r="E61" t="n">
         <v>3</v>
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.1696</v>
+        <v>0.1682</v>
       </c>
       <c r="E62" t="n">
         <v>1</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.1716</v>
+        <v>0.1733</v>
       </c>
       <c r="E63" t="n">
         <v>2</v>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.2196</v>
+        <v>0.2207</v>
       </c>
       <c r="E64" t="n">
         <v>3</v>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.3823</v>
+        <v>0.3824</v>
       </c>
       <c r="E65" t="n">
         <v>1</v>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.3846</v>
+        <v>0.3871</v>
       </c>
       <c r="E66" t="n">
         <v>2</v>
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.4123</v>
+        <v>0.4122</v>
       </c>
       <c r="E67" t="n">
         <v>3</v>
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.8072</v>
+        <v>0.8103</v>
       </c>
       <c r="E69" t="n">
         <v>2</v>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.9464</v>
+        <v>0.9479</v>
       </c>
       <c r="E70" t="n">
         <v>3</v>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.2068</v>
+        <v>0.2039</v>
       </c>
       <c r="E72" t="n">
         <v>2</v>
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.2375</v>
+        <v>0.2372</v>
       </c>
       <c r="E73" t="n">
         <v>3</v>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.6671</v>
+        <v>0.6685</v>
       </c>
       <c r="E75" t="n">
         <v>2</v>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.7547</v>
+        <v>0.7541</v>
       </c>
       <c r="E76" t="n">
         <v>3</v>
@@ -2605,7 +2605,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1.037</v>
+        <v>1.0396</v>
       </c>
       <c r="E78" t="n">
         <v>2</v>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.1996</v>
+        <v>1.2007</v>
       </c>
       <c r="E79" t="n">
         <v>3</v>
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.1016</v>
+        <v>0.1014</v>
       </c>
       <c r="E80" t="n">
         <v>1</v>
@@ -2689,7 +2689,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.1882</v>
+        <v>0.1909</v>
       </c>
       <c r="E81" t="n">
         <v>2</v>
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.2416</v>
+        <v>0.2408</v>
       </c>
       <c r="E82" t="n">
         <v>3</v>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.3046</v>
+        <v>0.308</v>
       </c>
       <c r="E83" t="n">
         <v>1</v>
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.3216</v>
+        <v>0.3106</v>
       </c>
       <c r="E84" t="n">
         <v>2</v>
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.853</v>
+        <v>0.8566</v>
       </c>
       <c r="E85" t="n">
         <v>3</v>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.5139</v>
+        <v>0.5144</v>
       </c>
       <c r="E86" t="n">
         <v>1</v>
@@ -2857,7 +2857,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.527</v>
+        <v>0.5264</v>
       </c>
       <c r="E87" t="n">
         <v>2</v>
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.5461</v>
+        <v>0.5469000000000001</v>
       </c>
       <c r="E88" t="n">
         <v>3</v>
@@ -2913,7 +2913,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.1155</v>
+        <v>0.1158</v>
       </c>
       <c r="E89" t="n">
         <v>1</v>
@@ -2941,7 +2941,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.3167</v>
+        <v>0.3111</v>
       </c>
       <c r="E90" t="n">
         <v>2</v>
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.3562</v>
+        <v>0.3565</v>
       </c>
       <c r="E91" t="n">
         <v>3</v>
@@ -2997,7 +2997,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.0813</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="E92" t="n">
         <v>1</v>
@@ -3025,7 +3025,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.0912</v>
+        <v>0.0911</v>
       </c>
       <c r="E93" t="n">
         <v>2</v>
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.0994</v>
+        <v>0.0993</v>
       </c>
       <c r="E94" t="n">
         <v>3</v>
@@ -3081,7 +3081,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.1523</v>
+        <v>0.1552</v>
       </c>
       <c r="E95" t="n">
         <v>1</v>
@@ -3109,7 +3109,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.2139</v>
+        <v>0.2133</v>
       </c>
       <c r="E96" t="n">
         <v>2</v>
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.316</v>
+        <v>0.3183</v>
       </c>
       <c r="E97" t="n">
         <v>3</v>
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>1.402</v>
+        <v>1.4332</v>
       </c>
       <c r="E98" t="n">
         <v>1</v>
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>1.8819</v>
+        <v>1.8896</v>
       </c>
       <c r="E99" t="n">
         <v>2</v>
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1.8954</v>
+        <v>1.9006</v>
       </c>
       <c r="E100" t="n">
         <v>3</v>
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>5.2368</v>
+        <v>5.2516</v>
       </c>
       <c r="E101" t="n">
         <v>1</v>
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>5.4799</v>
+        <v>5.4901</v>
       </c>
       <c r="E102" t="n">
         <v>2</v>
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>5.9826</v>
+        <v>5.9851</v>
       </c>
       <c r="E103" t="n">
         <v>3</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.5754</v>
+        <v>0.5749</v>
       </c>
       <c r="E104" t="n">
         <v>1</v>
@@ -3352,16 +3352,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>259960</t>
+          <t>035720</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>크래프톤</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.5913</v>
+        <v>0.5916</v>
       </c>
       <c r="E105" t="n">
         <v>2</v>
@@ -3380,16 +3380,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>259960</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>크래프톤</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.5916</v>
+        <v>0.5919</v>
       </c>
       <c r="E106" t="n">
         <v>3</v>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.1251</v>
+        <v>0.124</v>
       </c>
       <c r="E107" t="n">
         <v>1</v>
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.1537</v>
+        <v>0.1525</v>
       </c>
       <c r="E108" t="n">
         <v>2</v>
@@ -3473,7 +3473,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.2359</v>
+        <v>0.2397</v>
       </c>
       <c r="E109" t="n">
         <v>3</v>
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.2122</v>
+        <v>0.2128</v>
       </c>
       <c r="E110" t="n">
         <v>1</v>
@@ -3529,7 +3529,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.2214</v>
+        <v>0.2222</v>
       </c>
       <c r="E111" t="n">
         <v>2</v>
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.2427</v>
+        <v>0.2434</v>
       </c>
       <c r="E112" t="n">
         <v>3</v>
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.0746</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="E113" t="n">
         <v>1</v>
@@ -3613,7 +3613,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.0854</v>
       </c>
       <c r="E114" t="n">
         <v>2</v>
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0.1975</v>
+        <v>0.1962</v>
       </c>
       <c r="E117" t="n">
         <v>2</v>
@@ -3725,7 +3725,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.3513</v>
+        <v>0.3523</v>
       </c>
       <c r="E118" t="n">
         <v>3</v>
@@ -3753,7 +3753,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>1.9178</v>
+        <v>1.9195</v>
       </c>
       <c r="E119" t="n">
         <v>1</v>
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>2.011</v>
+        <v>2.0115</v>
       </c>
       <c r="E120" t="n">
         <v>2</v>
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>2.1289</v>
+        <v>2.1255</v>
       </c>
       <c r="E121" t="n">
         <v>3</v>
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.0593</v>
+        <v>0.0592</v>
       </c>
       <c r="E122" t="n">
         <v>1</v>
@@ -3865,7 +3865,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.0604</v>
+        <v>0.0612</v>
       </c>
       <c r="E123" t="n">
         <v>2</v>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0.0789</v>
+        <v>0.0796</v>
       </c>
       <c r="E124" t="n">
         <v>3</v>
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.1154</v>
+        <v>0.1153</v>
       </c>
       <c r="E126" t="n">
         <v>2</v>
@@ -3977,7 +3977,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0.1432</v>
+        <v>0.1401</v>
       </c>
       <c r="E127" t="n">
         <v>3</v>
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.2765</v>
+        <v>0.2784</v>
       </c>
       <c r="E128" t="n">
         <v>1</v>
@@ -4061,7 +4061,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0.4925</v>
+        <v>0.4909</v>
       </c>
       <c r="E130" t="n">
         <v>3</v>
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.8103</v>
+        <v>0.8109</v>
       </c>
       <c r="E131" t="n">
         <v>1</v>
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1.0176</v>
+        <v>1.02</v>
       </c>
       <c r="E132" t="n">
         <v>2</v>
@@ -4145,7 +4145,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1.1778</v>
+        <v>1.1788</v>
       </c>
       <c r="E133" t="n">
         <v>3</v>
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.094</v>
+        <v>0.0946</v>
       </c>
       <c r="E135" t="n">
         <v>2</v>
@@ -4229,7 +4229,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.0989</v>
+        <v>0.09959999999999999</v>
       </c>
       <c r="E136" t="n">
         <v>3</v>
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.3204</v>
+        <v>0.3272</v>
       </c>
       <c r="E137" t="n">
         <v>1</v>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.4697</v>
+        <v>0.4752</v>
       </c>
       <c r="E138" t="n">
         <v>2</v>
@@ -4313,7 +4313,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.5063</v>
+        <v>0.509</v>
       </c>
       <c r="E139" t="n">
         <v>3</v>
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.2686</v>
+        <v>0.2677</v>
       </c>
       <c r="E140" t="n">
         <v>1</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0.0762</v>
+        <v>0.076</v>
       </c>
       <c r="E143" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.0992</v>
+        <v>0.099</v>
       </c>
       <c r="E144" t="n">
         <v>2</v>
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.1396</v>
+        <v>0.1398</v>
       </c>
       <c r="E145" t="n">
         <v>3</v>
@@ -4509,7 +4509,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.1276</v>
+        <v>0.1225</v>
       </c>
       <c r="E146" t="n">
         <v>1</v>
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>0.3011</v>
+        <v>0.2988</v>
       </c>
       <c r="E147" t="n">
         <v>2</v>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0.4229</v>
+        <v>0.427</v>
       </c>
       <c r="E148" t="n">
         <v>3</v>
@@ -4593,7 +4593,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0.137</v>
+        <v>0.1374</v>
       </c>
       <c r="E149" t="n">
         <v>1</v>
@@ -4621,7 +4621,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.1516</v>
+        <v>0.1515</v>
       </c>
       <c r="E150" t="n">
         <v>2</v>
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.0786</v>
+        <v>0.0776</v>
       </c>
       <c r="E152" t="n">
         <v>1</v>
@@ -4733,7 +4733,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.1942</v>
+        <v>0.1926</v>
       </c>
       <c r="E154" t="n">
         <v>3</v>
@@ -4789,7 +4789,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>1.8806</v>
+        <v>1.8805</v>
       </c>
       <c r="E156" t="n">
         <v>2</v>
@@ -4845,7 +4845,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>7.9243</v>
+        <v>7.9237</v>
       </c>
       <c r="E158" t="n">
         <v>1</v>
@@ -4901,7 +4901,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>7.9652</v>
+        <v>7.9641</v>
       </c>
       <c r="E160" t="n">
         <v>3</v>
@@ -4929,7 +4929,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.3425</v>
+        <v>0.3293</v>
       </c>
       <c r="E161" t="n">
         <v>1</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.7846</v>
+        <v>0.7921</v>
       </c>
       <c r="E162" t="n">
         <v>2</v>
@@ -4985,7 +4985,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>0.9333</v>
+        <v>0.9368</v>
       </c>
       <c r="E163" t="n">
         <v>3</v>
@@ -5013,7 +5013,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>0.0448</v>
+        <v>0.0439</v>
       </c>
       <c r="E164" t="n">
         <v>1</v>
@@ -5069,7 +5069,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>0.1545</v>
+        <v>0.1542</v>
       </c>
       <c r="E166" t="n">
         <v>3</v>
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.1319</v>
+        <v>0.1365</v>
       </c>
       <c r="E167" t="n">
         <v>1</v>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0.1374</v>
+        <v>0.1369</v>
       </c>
       <c r="E168" t="n">
         <v>2</v>
@@ -5181,7 +5181,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.2079</v>
+        <v>0.2106</v>
       </c>
       <c r="E170" t="n">
         <v>1</v>
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0.3145</v>
+        <v>0.316</v>
       </c>
       <c r="E171" t="n">
         <v>2</v>
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0.3177</v>
+        <v>0.3185</v>
       </c>
       <c r="E172" t="n">
         <v>3</v>
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>0.0399</v>
+        <v>0.0384</v>
       </c>
       <c r="E173" t="n">
         <v>1</v>
@@ -5321,7 +5321,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>0.0989</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="E175" t="n">
         <v>3</v>
@@ -5349,7 +5349,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>0.0573</v>
+        <v>0.0595</v>
       </c>
       <c r="E176" t="n">
         <v>1</v>
@@ -5377,7 +5377,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>0.1088</v>
+        <v>0.107</v>
       </c>
       <c r="E177" t="n">
         <v>2</v>
@@ -5433,7 +5433,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>0.4167</v>
+        <v>0.4129</v>
       </c>
       <c r="E179" t="n">
         <v>1</v>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>1.1399</v>
+        <v>1.1426</v>
       </c>
       <c r="E180" t="n">
         <v>2</v>
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>1.2856</v>
+        <v>1.2886</v>
       </c>
       <c r="E181" t="n">
         <v>3</v>
@@ -5517,7 +5517,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.0634</v>
       </c>
       <c r="E182" t="n">
         <v>1</v>
@@ -5545,7 +5545,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.0709</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="E183" t="n">
         <v>2</v>
@@ -5573,7 +5573,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>0.0764</v>
+        <v>0.077</v>
       </c>
       <c r="E184" t="n">
         <v>3</v>
@@ -5629,7 +5629,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.0897</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="E186" t="n">
         <v>2</v>
@@ -5657,7 +5657,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0.1066</v>
+        <v>0.1068</v>
       </c>
       <c r="E187" t="n">
         <v>3</v>
@@ -5685,7 +5685,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>1.2195</v>
+        <v>1.2318</v>
       </c>
       <c r="E188" t="n">
         <v>1</v>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>2.155</v>
+        <v>2.1622</v>
       </c>
       <c r="E189" t="n">
         <v>2</v>
@@ -5741,7 +5741,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>2.2576</v>
+        <v>2.2612</v>
       </c>
       <c r="E190" t="n">
         <v>3</v>
@@ -5825,7 +5825,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>0.1927</v>
+        <v>0.1891</v>
       </c>
       <c r="E193" t="n">
         <v>3</v>
@@ -5853,7 +5853,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>0.1143</v>
+        <v>0.1136</v>
       </c>
       <c r="E194" t="n">
         <v>1</v>
@@ -5881,7 +5881,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>0.1169</v>
+        <v>0.1153</v>
       </c>
       <c r="E195" t="n">
         <v>2</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>0.1731</v>
+        <v>0.1734</v>
       </c>
       <c r="E196" t="n">
         <v>3</v>
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>0.0554</v>
+        <v>0.0538</v>
       </c>
       <c r="E197" t="n">
         <v>1</v>
@@ -5965,7 +5965,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>0.1364</v>
+        <v>0.1384</v>
       </c>
       <c r="E198" t="n">
         <v>2</v>
@@ -5993,7 +5993,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>0.1509</v>
+        <v>0.1477</v>
       </c>
       <c r="E199" t="n">
         <v>3</v>
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>0.1316</v>
+        <v>0.132</v>
       </c>
       <c r="E200" t="n">
         <v>1</v>
@@ -6049,7 +6049,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>0.158</v>
+        <v>0.1587</v>
       </c>
       <c r="E201" t="n">
         <v>2</v>
@@ -6105,7 +6105,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>0.0116</v>
+        <v>0.0122</v>
       </c>
       <c r="E203" t="n">
         <v>1</v>
@@ -6133,7 +6133,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>0.0152</v>
+        <v>0.0156</v>
       </c>
       <c r="E204" t="n">
         <v>2</v>
@@ -6161,7 +6161,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>0.0406</v>
+        <v>0.0403</v>
       </c>
       <c r="E205" t="n">
         <v>3</v>
@@ -6189,7 +6189,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>0.0834</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="E206" t="n">
         <v>1</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>0.2117</v>
+        <v>0.2098</v>
       </c>
       <c r="E208" t="n">
         <v>3</v>
@@ -6273,7 +6273,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>0.0225</v>
+        <v>0.0226</v>
       </c>
       <c r="E209" t="n">
         <v>1</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>0.0339</v>
+        <v>0.0335</v>
       </c>
       <c r="E210" t="n">
         <v>2</v>
@@ -6329,7 +6329,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>0.0346</v>
+        <v>0.0342</v>
       </c>
       <c r="E211" t="n">
         <v>3</v>
@@ -6357,7 +6357,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>0.1318</v>
+        <v>0.1373</v>
       </c>
       <c r="E212" t="n">
         <v>1</v>
@@ -6385,7 +6385,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>0.1632</v>
+        <v>0.1673</v>
       </c>
       <c r="E213" t="n">
         <v>2</v>
@@ -6413,7 +6413,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>0.2018</v>
+        <v>0.2033</v>
       </c>
       <c r="E214" t="n">
         <v>3</v>
@@ -6441,7 +6441,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>0.0137</v>
+        <v>0.0133</v>
       </c>
       <c r="E215" t="n">
         <v>1</v>
@@ -6469,7 +6469,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>0.0284</v>
+        <v>0.0278</v>
       </c>
       <c r="E216" t="n">
         <v>2</v>
@@ -6525,7 +6525,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>0.0141</v>
+        <v>0.0145</v>
       </c>
       <c r="E218" t="n">
         <v>1</v>
@@ -6553,7 +6553,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>0.0396</v>
+        <v>0.0403</v>
       </c>
       <c r="E219" t="n">
         <v>2</v>
@@ -6609,7 +6609,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>0.1224</v>
+        <v>0.1193</v>
       </c>
       <c r="E221" t="n">
         <v>1</v>
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>0.1492</v>
+        <v>0.1473</v>
       </c>
       <c r="E222" t="n">
         <v>2</v>
@@ -6665,7 +6665,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>0.1633</v>
+        <v>0.1662</v>
       </c>
       <c r="E223" t="n">
         <v>3</v>
@@ -6693,7 +6693,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>0.105</v>
+        <v>0.1052</v>
       </c>
       <c r="E224" t="n">
         <v>1</v>
@@ -6721,7 +6721,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>0.1513</v>
+        <v>0.1518</v>
       </c>
       <c r="E225" t="n">
         <v>2</v>
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>0.1611</v>
+        <v>0.161</v>
       </c>
       <c r="E226" t="n">
         <v>3</v>
@@ -6777,7 +6777,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>0.0696</v>
+        <v>0.0694</v>
       </c>
       <c r="E227" t="n">
         <v>1</v>
@@ -6833,7 +6833,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>0.1625</v>
+        <v>0.1628</v>
       </c>
       <c r="E229" t="n">
         <v>3</v>
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0.0391</v>
+        <v>0.0401</v>
       </c>
       <c r="E230" t="n">
         <v>1</v>
@@ -6889,7 +6889,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0.0737</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="E231" t="n">
         <v>2</v>
@@ -6917,7 +6917,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0.0929</v>
+        <v>0.0992</v>
       </c>
       <c r="E232" t="n">
         <v>3</v>
@@ -6945,7 +6945,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>0.0524</v>
+        <v>0.0491</v>
       </c>
       <c r="E233" t="n">
         <v>1</v>
@@ -6973,7 +6973,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>0.0622</v>
+        <v>0.0635</v>
       </c>
       <c r="E234" t="n">
         <v>2</v>
@@ -7029,7 +7029,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>0.7457</v>
+        <v>0.7481</v>
       </c>
       <c r="E236" t="n">
         <v>1</v>
@@ -7085,7 +7085,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>0.9426</v>
+        <v>0.9431</v>
       </c>
       <c r="E238" t="n">
         <v>3</v>
@@ -7113,7 +7113,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>0.0578</v>
+        <v>0.058</v>
       </c>
       <c r="E239" t="n">
         <v>1</v>
@@ -7141,7 +7141,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>0.1135</v>
+        <v>0.1136</v>
       </c>
       <c r="E240" t="n">
         <v>2</v>
@@ -7169,7 +7169,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>0.1238</v>
+        <v>0.1234</v>
       </c>
       <c r="E241" t="n">
         <v>3</v>
@@ -7197,7 +7197,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>0.1787</v>
+        <v>0.1784</v>
       </c>
       <c r="E242" t="n">
         <v>1</v>
@@ -7225,7 +7225,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>0.2039</v>
+        <v>0.2059</v>
       </c>
       <c r="E243" t="n">
         <v>2</v>
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>0.3378</v>
+        <v>0.3387</v>
       </c>
       <c r="E244" t="n">
         <v>3</v>
@@ -7309,7 +7309,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>0.3955</v>
+        <v>0.3964</v>
       </c>
       <c r="E246" t="n">
         <v>2</v>
@@ -7337,7 +7337,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>0.3991</v>
+        <v>0.4017</v>
       </c>
       <c r="E247" t="n">
         <v>3</v>
@@ -7393,7 +7393,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>0.4077</v>
+        <v>0.4104</v>
       </c>
       <c r="E249" t="n">
         <v>2</v>
@@ -7421,7 +7421,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>0.4151</v>
+        <v>0.4161</v>
       </c>
       <c r="E250" t="n">
         <v>3</v>
@@ -7449,7 +7449,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>0.7674</v>
+        <v>0.764</v>
       </c>
       <c r="E251" t="n">
         <v>1</v>
@@ -7477,7 +7477,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>1.0917</v>
+        <v>1.0939</v>
       </c>
       <c r="E252" t="n">
         <v>2</v>
@@ -7505,7 +7505,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>1.3221</v>
+        <v>1.3232</v>
       </c>
       <c r="E253" t="n">
         <v>3</v>
@@ -7533,7 +7533,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>0.0343</v>
+        <v>0.0345</v>
       </c>
       <c r="E254" t="n">
         <v>1</v>
@@ -7561,7 +7561,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>0.0362</v>
+        <v>0.0351</v>
       </c>
       <c r="E255" t="n">
         <v>2</v>
@@ -7589,7 +7589,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>0.0446</v>
+        <v>0.0451</v>
       </c>
       <c r="E256" t="n">
         <v>3</v>
@@ -7617,7 +7617,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>0.0288</v>
+        <v>0.0289</v>
       </c>
       <c r="E257" t="n">
         <v>1</v>
@@ -7645,7 +7645,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>0.0389</v>
+        <v>0.0386</v>
       </c>
       <c r="E258" t="n">
         <v>2</v>
@@ -7673,7 +7673,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>0.0574</v>
+        <v>0.0578</v>
       </c>
       <c r="E259" t="n">
         <v>3</v>
@@ -7701,7 +7701,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>0.4037</v>
+        <v>0.4016</v>
       </c>
       <c r="E260" t="n">
         <v>1</v>
@@ -7729,7 +7729,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>0.5595</v>
+        <v>0.5579</v>
       </c>
       <c r="E261" t="n">
         <v>2</v>
@@ -7757,7 +7757,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>0.6296</v>
+        <v>0.632</v>
       </c>
       <c r="E262" t="n">
         <v>3</v>
@@ -7785,7 +7785,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>0.8075</v>
+        <v>0.8102</v>
       </c>
       <c r="E263" t="n">
         <v>1</v>
@@ -7841,7 +7841,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>1.0554</v>
+        <v>1.0537</v>
       </c>
       <c r="E265" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Update README with full feature table, evaluation results, and DART setup; bump theme weight to 3x
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -468,12 +468,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>055550</t>
+          <t>329180</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -496,16 +496,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>034020</t>
+          <t>010130</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>고려아연</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4.3623</v>
+        <v>4.5996</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -524,16 +524,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>079550</t>
+          <t>316140</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LIG디펜스앤에어로스페이스</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4.5986</v>
+        <v>4.6741</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.1804</v>
+        <v>2.1813</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.5679</v>
+        <v>2.5689</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -608,12 +608,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -636,12 +636,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.566</v>
+        <v>1.5616</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -692,16 +692,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>000660</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.8915</v>
+        <v>1.9146</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5.2385</v>
+        <v>5.2391</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -776,12 +776,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -804,12 +804,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>090430</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8.7784</v>
+        <v>12.4804</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
@@ -860,16 +860,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8.9132</v>
+        <v>12.5755</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -888,12 +888,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>090430</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8.447699999999999</v>
+        <v>12.25</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
@@ -944,16 +944,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8.510999999999999</v>
+        <v>12.2937</v>
       </c>
       <c r="E19" t="n">
         <v>3</v>
@@ -981,7 +981,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2.3533</v>
+        <v>2.3541</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
@@ -1000,12 +1000,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3.5364</v>
+        <v>3.5345</v>
       </c>
       <c r="E22" t="n">
         <v>3</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6.2704</v>
+        <v>9.2212</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -1084,16 +1084,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6.2765</v>
+        <v>9.225199999999999</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -1112,16 +1112,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6.3941</v>
+        <v>9.3057</v>
       </c>
       <c r="E25" t="n">
         <v>3</v>
@@ -1140,16 +1140,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>017670</t>
+          <t>015760</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>한국전력</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3.1859</v>
+        <v>3.1858</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
@@ -1168,12 +1168,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>011070</t>
+          <t>009540</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1196,16 +1196,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>086280</t>
+          <t>010140</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>현대글로비스</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.2222</v>
+        <v>3.2221</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -1224,16 +1224,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>207940</t>
+          <t>032830</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.0251</v>
+        <v>1.0357</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
@@ -1252,16 +1252,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>298040</t>
+          <t>086790</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2.2663</v>
+        <v>2.9221</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
@@ -1280,16 +1280,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>028260</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2.9205</v>
+        <v>2.9537</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
@@ -1308,16 +1308,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>307950</t>
+          <t>011200</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>현대오토에버</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.5204</v>
+        <v>0.5203</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
@@ -1336,12 +1336,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>066570</t>
+          <t>267260</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>HD현대일렉트릭</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1364,16 +1364,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>316140</t>
+          <t>000810</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.672</v>
+        <v>0.6719000000000001</v>
       </c>
       <c r="E34" t="n">
         <v>3</v>
@@ -1392,16 +1392,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>005930</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>8.235900000000001</v>
+        <v>10.6747</v>
       </c>
       <c r="E35" t="n">
         <v>1</v>
@@ -1420,16 +1420,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>009150</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8.260400000000001</v>
+        <v>10.7322</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -1448,16 +1448,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>000660</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8.314500000000001</v>
+        <v>10.7981</v>
       </c>
       <c r="E37" t="n">
         <v>3</v>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4.7088</v>
+        <v>4.7091</v>
       </c>
       <c r="E38" t="n">
         <v>1</v>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5.6252</v>
+        <v>5.6249</v>
       </c>
       <c r="E39" t="n">
         <v>2</v>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1560,16 +1560,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.6319</v>
+        <v>0.8615</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
@@ -1588,23 +1588,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.8617</v>
+        <v>1.5197</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -1616,23 +1616,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>033780</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1.4333</v>
+        <v>10.6476</v>
       </c>
       <c r="E43" t="n">
         <v>3</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -1644,12 +1644,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>267260</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1672,16 +1672,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>298040</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>5.9682</v>
+        <v>6.0091</v>
       </c>
       <c r="E45" t="n">
         <v>2</v>
@@ -1700,16 +1700,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>105560</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>6.0091</v>
+        <v>6.3607</v>
       </c>
       <c r="E46" t="n">
         <v>3</v>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.5576</v>
+        <v>0.5996</v>
       </c>
       <c r="E47" t="n">
         <v>1</v>
@@ -1756,16 +1756,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>267260</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.5985</v>
+        <v>0.7086</v>
       </c>
       <c r="E48" t="n">
         <v>2</v>
@@ -1784,16 +1784,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>028260</t>
+          <t>105560</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.6308</v>
+        <v>0.7979000000000001</v>
       </c>
       <c r="E49" t="n">
         <v>3</v>
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.4218</v>
+        <v>1.4227</v>
       </c>
       <c r="E50" t="n">
         <v>1</v>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3.2366</v>
+        <v>3.2361</v>
       </c>
       <c r="E51" t="n">
         <v>2</v>
@@ -1868,12 +1868,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1896,16 +1896,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.6331</v>
+        <v>0.6326000000000001</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
@@ -1924,23 +1924,23 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>033780</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.9847</v>
+        <v>1.8653</v>
       </c>
       <c r="E54" t="n">
         <v>2</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -1952,23 +1952,23 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>005380</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1.0677</v>
+        <v>10.7313</v>
       </c>
       <c r="E55" t="n">
         <v>3</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -1980,16 +1980,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>6.9083</v>
+        <v>9.666399999999999</v>
       </c>
       <c r="E56" t="n">
         <v>1</v>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>6.9204</v>
+        <v>9.675000000000001</v>
       </c>
       <c r="E57" t="n">
         <v>2</v>
@@ -2036,16 +2036,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>7.1122</v>
+        <v>9.8131</v>
       </c>
       <c r="E58" t="n">
         <v>3</v>
@@ -2064,12 +2064,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2148,12 +2148,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>090430</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2176,16 +2176,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>8.447100000000001</v>
+        <v>12.2496</v>
       </c>
       <c r="E63" t="n">
         <v>2</v>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>8.5251</v>
+        <v>12.3035</v>
       </c>
       <c r="E64" t="n">
         <v>3</v>
@@ -2232,16 +2232,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>011070</t>
+          <t>009540</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.8627</v>
+        <v>0.8621</v>
       </c>
       <c r="E65" t="n">
         <v>1</v>
@@ -2260,16 +2260,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>034020</t>
+          <t>010130</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>고려아연</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1.0862</v>
+        <v>1.2423</v>
       </c>
       <c r="E66" t="n">
         <v>2</v>
@@ -2288,16 +2288,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>079550</t>
+          <t>316140</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LIG디펜스앤에어로스페이스</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1.2421</v>
+        <v>1.2771</v>
       </c>
       <c r="E67" t="n">
         <v>3</v>
@@ -2316,23 +2316,23 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.3431</v>
+        <v>1.6346</v>
       </c>
       <c r="E68" t="n">
         <v>1</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -2344,16 +2344,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1.6369</v>
+        <v>1.6759</v>
       </c>
       <c r="E69" t="n">
         <v>2</v>
@@ -2372,16 +2372,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>028260</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1.6535</v>
+        <v>1.7055</v>
       </c>
       <c r="E70" t="n">
         <v>3</v>
@@ -2400,16 +2400,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>015760</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>한국전력</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.7772</v>
+        <v>0.8925</v>
       </c>
       <c r="E71" t="n">
         <v>1</v>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.7947</v>
+        <v>0.9255</v>
       </c>
       <c r="E72" t="n">
         <v>2</v>
@@ -2456,16 +2456,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>030200</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.8924</v>
+        <v>0.9849</v>
       </c>
       <c r="E73" t="n">
         <v>3</v>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>6.4677</v>
+        <v>9.3565</v>
       </c>
       <c r="E74" t="n">
         <v>1</v>
@@ -2512,16 +2512,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6.5921</v>
+        <v>9.4429</v>
       </c>
       <c r="E75" t="n">
         <v>2</v>
@@ -2540,16 +2540,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>6.6744</v>
+        <v>9.500500000000001</v>
       </c>
       <c r="E76" t="n">
         <v>3</v>
@@ -2568,16 +2568,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1.1871</v>
+        <v>1.4153</v>
       </c>
       <c r="E77" t="n">
         <v>1</v>
@@ -2596,16 +2596,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>267260</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1.4142</v>
+        <v>1.4745</v>
       </c>
       <c r="E78" t="n">
         <v>2</v>
@@ -2624,23 +2624,23 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>028260</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.4344</v>
+        <v>1.5134</v>
       </c>
       <c r="E79" t="n">
         <v>3</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -2652,16 +2652,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>011070</t>
+          <t>009540</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.6913</v>
+        <v>0.6906</v>
       </c>
       <c r="E80" t="n">
         <v>1</v>
@@ -2680,16 +2680,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>079550</t>
+          <t>010130</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LIG디펜스앤에어로스페이스</t>
+          <t>고려아연</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1.2381</v>
+        <v>1.2382</v>
       </c>
       <c r="E81" t="n">
         <v>2</v>
@@ -2708,23 +2708,23 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>005940</t>
+          <t>015760</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>한국전력</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.3175</v>
+        <v>1.5478</v>
       </c>
       <c r="E82" t="n">
         <v>3</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -2736,16 +2736,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>062040</t>
+          <t>034730</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>산일전기</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1.9502</v>
+        <v>2.5743</v>
       </c>
       <c r="E83" t="n">
         <v>1</v>
@@ -2764,16 +2764,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>086790</t>
+          <t>028260</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>2.5745</v>
+        <v>2.6427</v>
       </c>
       <c r="E84" t="n">
         <v>2</v>
@@ -2792,16 +2792,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>000270</t>
+          <t>272210</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>2.6423</v>
+        <v>2.6561</v>
       </c>
       <c r="E85" t="n">
         <v>3</v>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>6.124</v>
+        <v>9.122400000000001</v>
       </c>
       <c r="E86" t="n">
         <v>1</v>
@@ -2848,16 +2848,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>6.1995</v>
+        <v>9.1731</v>
       </c>
       <c r="E87" t="n">
         <v>2</v>
@@ -2876,16 +2876,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>6.2295</v>
+        <v>9.1935</v>
       </c>
       <c r="E88" t="n">
         <v>3</v>
@@ -2904,16 +2904,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>005380</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.5393</v>
+        <v>0.6764</v>
       </c>
       <c r="E89" t="n">
         <v>1</v>
@@ -2932,23 +2932,23 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.677</v>
+        <v>2.0242</v>
       </c>
       <c r="E90" t="n">
         <v>2</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -2960,23 +2960,23 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>033780</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1.2773</v>
+        <v>10.7533</v>
       </c>
       <c r="E91" t="n">
         <v>3</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -2988,12 +2988,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3016,12 +3016,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -3044,16 +3044,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>1.2387</v>
+        <v>1.2385</v>
       </c>
       <c r="E94" t="n">
         <v>3</v>
@@ -3072,12 +3072,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2.7646</v>
+        <v>2.7644</v>
       </c>
       <c r="E97" t="n">
         <v>3</v>
@@ -3156,16 +3156,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>024110</t>
+          <t>316140</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>기업은행</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>2.5246</v>
+        <v>2.5223</v>
       </c>
       <c r="E98" t="n">
         <v>1</v>
@@ -3184,16 +3184,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>011200</t>
+          <t>006800</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>2.8842</v>
+        <v>2.8825</v>
       </c>
       <c r="E99" t="n">
         <v>2</v>
@@ -3212,12 +3212,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>055550</t>
+          <t>329180</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>6.1903</v>
+        <v>6.1995</v>
       </c>
       <c r="E101" t="n">
         <v>1</v>
@@ -3268,16 +3268,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>042660</t>
+          <t>000660</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>6.9085</v>
+        <v>7.3011</v>
       </c>
       <c r="E102" t="n">
         <v>2</v>
@@ -3296,16 +3296,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>000660</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>7.3001</v>
+        <v>7.3782</v>
       </c>
       <c r="E103" t="n">
         <v>3</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>6.2589</v>
+        <v>9.2135</v>
       </c>
       <c r="E104" t="n">
         <v>1</v>
@@ -3352,16 +3352,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>6.3256</v>
+        <v>9.258900000000001</v>
       </c>
       <c r="E105" t="n">
         <v>2</v>
@@ -3380,16 +3380,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>6.3773</v>
+        <v>9.2943</v>
       </c>
       <c r="E106" t="n">
         <v>3</v>
@@ -3408,16 +3408,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>011200</t>
+          <t>006800</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.9832</v>
+        <v>0.9829</v>
       </c>
       <c r="E107" t="n">
         <v>1</v>
@@ -3436,16 +3436,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>000880</t>
+          <t>018260</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>삼성에스디에스</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1.1239</v>
+        <v>1.124</v>
       </c>
       <c r="E108" t="n">
         <v>2</v>
@@ -3464,16 +3464,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>017670</t>
+          <t>015760</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>한국전력</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1.1719</v>
+        <v>1.1715</v>
       </c>
       <c r="E109" t="n">
         <v>3</v>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>090430</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3520,16 +3520,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>8.0329</v>
+        <v>11.9677</v>
       </c>
       <c r="E111" t="n">
         <v>2</v>
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>8.2028</v>
+        <v>12.0825</v>
       </c>
       <c r="E112" t="n">
         <v>3</v>
@@ -3576,12 +3576,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3604,12 +3604,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3660,16 +3660,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>1.0626</v>
+        <v>1.0611</v>
       </c>
       <c r="E116" t="n">
         <v>1</v>
@@ -3688,16 +3688,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>1.1208</v>
+        <v>1.1619</v>
       </c>
       <c r="E117" t="n">
         <v>2</v>
@@ -3716,16 +3716,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>267260</t>
+          <t>105560</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1.1614</v>
+        <v>1.4969</v>
       </c>
       <c r="E118" t="n">
         <v>3</v>
@@ -3744,16 +3744,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>033780</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>2.3876</v>
+        <v>2.8481</v>
       </c>
       <c r="E119" t="n">
         <v>1</v>
@@ -3772,23 +3772,23 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>005380</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>2.4077</v>
+        <v>3.8087</v>
       </c>
       <c r="E120" t="n">
         <v>2</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>⚠</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -3800,23 +3800,23 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>2.8485</v>
+        <v>11.2117</v>
       </c>
       <c r="E121" t="n">
         <v>3</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>⚠</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -3828,12 +3828,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>090430</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3856,16 +3856,16 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>7.9924</v>
+        <v>11.9406</v>
       </c>
       <c r="E123" t="n">
         <v>2</v>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>8.052</v>
+        <v>11.9806</v>
       </c>
       <c r="E124" t="n">
         <v>3</v>
@@ -3912,12 +3912,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3940,16 +3940,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>018260</t>
+          <t>042700</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>삼성에스디에스</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.6163</v>
+        <v>0.616</v>
       </c>
       <c r="E126" t="n">
         <v>2</v>
@@ -3968,16 +3968,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>161390</t>
+          <t>011200</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0.6576</v>
+        <v>0.8199</v>
       </c>
       <c r="E127" t="n">
         <v>3</v>
@@ -3996,16 +3996,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>010120</t>
+          <t>086790</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>LS ELECTRIC</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.7207</v>
+        <v>0.7204</v>
       </c>
       <c r="E128" t="n">
         <v>1</v>
@@ -4024,12 +4024,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -4052,12 +4052,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>005490</t>
+          <t>035420</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>NAVER</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>6.5576</v>
+        <v>9.418799999999999</v>
       </c>
       <c r="E131" t="n">
         <v>1</v>
@@ -4108,16 +4108,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>6.6281</v>
+        <v>9.4679</v>
       </c>
       <c r="E132" t="n">
         <v>2</v>
@@ -4136,16 +4136,16 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>6.7077</v>
+        <v>9.523899999999999</v>
       </c>
       <c r="E133" t="n">
         <v>3</v>
@@ -4164,12 +4164,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>090430</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>8.6311</v>
+        <v>12.3772</v>
       </c>
       <c r="E135" t="n">
         <v>2</v>
@@ -4220,16 +4220,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>8.7027</v>
+        <v>12.4272</v>
       </c>
       <c r="E136" t="n">
         <v>3</v>
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1.0958</v>
+        <v>1.09</v>
       </c>
       <c r="E137" t="n">
         <v>1</v>
@@ -4276,16 +4276,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>1.8943</v>
+        <v>1.973</v>
       </c>
       <c r="E138" t="n">
         <v>2</v>
@@ -4304,16 +4304,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>042660</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>1.973</v>
+        <v>2.5797</v>
       </c>
       <c r="E139" t="n">
         <v>3</v>
@@ -4332,12 +4332,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4369,7 +4369,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>2.6663</v>
+        <v>2.6664</v>
       </c>
       <c r="E141" t="n">
         <v>2</v>
@@ -4397,7 +4397,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>2.7033</v>
+        <v>2.7031</v>
       </c>
       <c r="E142" t="n">
         <v>3</v>
@@ -4416,12 +4416,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>2.4722</v>
+        <v>2.4723</v>
       </c>
       <c r="E144" t="n">
         <v>2</v>
@@ -4472,16 +4472,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>2.6101</v>
+        <v>2.61</v>
       </c>
       <c r="E145" t="n">
         <v>3</v>
@@ -4500,16 +4500,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>161390</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>1.099</v>
+        <v>1.1521</v>
       </c>
       <c r="E146" t="n">
         <v>1</v>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>1.1156</v>
+        <v>1.2423</v>
       </c>
       <c r="E147" t="n">
         <v>2</v>
@@ -4556,16 +4556,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>042700</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>1.1523</v>
+        <v>1.2791</v>
       </c>
       <c r="E148" t="n">
         <v>3</v>
@@ -4584,12 +4584,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4612,16 +4612,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>1.3031</v>
+        <v>1.303</v>
       </c>
       <c r="E150" t="n">
         <v>2</v>
@@ -4640,16 +4640,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>1.5356</v>
+        <v>1.5355</v>
       </c>
       <c r="E151" t="n">
         <v>3</v>
@@ -4668,12 +4668,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>2.3807</v>
+        <v>2.3805</v>
       </c>
       <c r="E153" t="n">
         <v>2</v>
@@ -4724,16 +4724,16 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>2.3873</v>
+        <v>2.3875</v>
       </c>
       <c r="E154" t="n">
         <v>3</v>
@@ -4789,7 +4789,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>2.41</v>
+        <v>2.4098</v>
       </c>
       <c r="E156" t="n">
         <v>2</v>
@@ -4808,12 +4808,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -4836,12 +4836,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -4864,16 +4864,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>7.9328</v>
+        <v>7.9334</v>
       </c>
       <c r="E159" t="n">
         <v>2</v>
@@ -4892,12 +4892,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>035420</t>
+          <t>042660</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4929,7 +4929,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>1.3327</v>
+        <v>1.3319</v>
       </c>
       <c r="E161" t="n">
         <v>1</v>
@@ -4948,12 +4948,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4976,16 +4976,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>005930</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>2.4009</v>
+        <v>2.6375</v>
       </c>
       <c r="E163" t="n">
         <v>3</v>
@@ -5004,23 +5004,23 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>1.3047</v>
+        <v>1.6782</v>
       </c>
       <c r="E164" t="n">
         <v>1</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -5032,16 +5032,16 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>033780</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>1.5376</v>
+        <v>2.2179</v>
       </c>
       <c r="E165" t="n">
         <v>2</v>
@@ -5060,23 +5060,23 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>1.6779</v>
+        <v>10.7958</v>
       </c>
       <c r="E166" t="n">
         <v>3</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>⚠</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -5088,16 +5088,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>003550</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.6581</v>
+        <v>0.658</v>
       </c>
       <c r="E167" t="n">
         <v>1</v>
@@ -5116,16 +5116,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0.7697000000000001</v>
+        <v>0.9825</v>
       </c>
       <c r="E168" t="n">
         <v>2</v>
@@ -5144,23 +5144,23 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>0.9824000000000001</v>
+        <v>10.4976</v>
       </c>
       <c r="E169" t="n">
         <v>3</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -5172,12 +5172,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>2.0504</v>
+        <v>2.0448</v>
       </c>
       <c r="E171" t="n">
         <v>2</v>
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>2.0986</v>
+        <v>2.099</v>
       </c>
       <c r="E172" t="n">
         <v>3</v>
@@ -5256,16 +5256,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>0.8855</v>
+        <v>1.3005</v>
       </c>
       <c r="E173" t="n">
         <v>1</v>
@@ -5284,23 +5284,23 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>1.3003</v>
+        <v>1.7753</v>
       </c>
       <c r="E174" t="n">
         <v>2</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -5312,23 +5312,23 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>033780</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>1.4359</v>
+        <v>10.7022</v>
       </c>
       <c r="E175" t="n">
         <v>3</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -5340,12 +5340,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -5368,12 +5368,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -5396,16 +5396,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>2.0267</v>
+        <v>2.0265</v>
       </c>
       <c r="E178" t="n">
         <v>3</v>
@@ -5424,12 +5424,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>2.026</v>
+        <v>2.023</v>
       </c>
       <c r="E180" t="n">
         <v>2</v>
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>2.15</v>
+        <v>2.1512</v>
       </c>
       <c r="E181" t="n">
         <v>3</v>
@@ -5517,7 +5517,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>6.4954</v>
+        <v>9.3758</v>
       </c>
       <c r="E182" t="n">
         <v>1</v>
@@ -5536,16 +5536,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>6.6107</v>
+        <v>9.456</v>
       </c>
       <c r="E183" t="n">
         <v>2</v>
@@ -5564,16 +5564,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>6.6249</v>
+        <v>9.4659</v>
       </c>
       <c r="E184" t="n">
         <v>3</v>
@@ -5592,16 +5592,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0.7702</v>
+        <v>0.7701</v>
       </c>
       <c r="E185" t="n">
         <v>1</v>
@@ -5620,16 +5620,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.868</v>
+        <v>0.8679</v>
       </c>
       <c r="E186" t="n">
         <v>2</v>
@@ -5648,16 +5648,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>015760</t>
+          <t>030200</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>한국전력</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>1.0235</v>
+        <v>1.0434</v>
       </c>
       <c r="E187" t="n">
         <v>3</v>
@@ -5685,7 +5685,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>3.1352</v>
+        <v>3.1393</v>
       </c>
       <c r="E188" t="n">
         <v>1</v>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3.4352</v>
+        <v>3.436</v>
       </c>
       <c r="E189" t="n">
         <v>2</v>
@@ -5732,12 +5732,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -5760,12 +5760,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -5825,7 +5825,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>2.4671</v>
+        <v>2.4669</v>
       </c>
       <c r="E193" t="n">
         <v>3</v>
@@ -5844,16 +5844,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>0.5429</v>
+        <v>0.5424</v>
       </c>
       <c r="E194" t="n">
         <v>1</v>
@@ -5872,16 +5872,16 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>0.8179</v>
+        <v>0.8181</v>
       </c>
       <c r="E195" t="n">
         <v>2</v>
@@ -5900,16 +5900,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>035420</t>
+          <t>042660</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>1.118</v>
+        <v>1.1182</v>
       </c>
       <c r="E196" t="n">
         <v>3</v>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>0.4577</v>
+        <v>0.4576</v>
       </c>
       <c r="E197" t="n">
         <v>1</v>
@@ -5956,12 +5956,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>066570</t>
+          <t>267260</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>LG전자</t>
+          <t>HD현대일렉트릭</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -5984,16 +5984,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>018260</t>
+          <t>042700</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>삼성에스디에스</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>0.5488</v>
+        <v>0.5486</v>
       </c>
       <c r="E199" t="n">
         <v>3</v>
@@ -6012,12 +6012,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -6068,16 +6068,16 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>2.6375</v>
+        <v>2.6374</v>
       </c>
       <c r="E202" t="n">
         <v>3</v>
@@ -6105,7 +6105,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>6.084</v>
+        <v>9.095599999999999</v>
       </c>
       <c r="E203" t="n">
         <v>1</v>
@@ -6124,16 +6124,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>6.1343</v>
+        <v>9.129300000000001</v>
       </c>
       <c r="E204" t="n">
         <v>2</v>
@@ -6152,16 +6152,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>6.1546</v>
+        <v>9.142899999999999</v>
       </c>
       <c r="E205" t="n">
         <v>3</v>
@@ -6180,12 +6180,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -6208,16 +6208,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>2.0592</v>
+        <v>2.0593</v>
       </c>
       <c r="E207" t="n">
         <v>2</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2.1459</v>
+        <v>2.1457</v>
       </c>
       <c r="E208" t="n">
         <v>3</v>
@@ -6273,7 +6273,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6.5486</v>
+        <v>9.412699999999999</v>
       </c>
       <c r="E209" t="n">
         <v>1</v>
@@ -6292,16 +6292,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>6.6511</v>
+        <v>9.484299999999999</v>
       </c>
       <c r="E210" t="n">
         <v>2</v>
@@ -6320,16 +6320,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>6.7636</v>
+        <v>9.563499999999999</v>
       </c>
       <c r="E211" t="n">
         <v>3</v>
@@ -6348,16 +6348,16 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>0.397</v>
+        <v>0.6227</v>
       </c>
       <c r="E212" t="n">
         <v>1</v>
@@ -6376,16 +6376,16 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>161390</t>
+          <t>105560</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>0.5587</v>
+        <v>0.6299</v>
       </c>
       <c r="E213" t="n">
         <v>2</v>
@@ -6404,16 +6404,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>028260</t>
+          <t>086790</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>0.5697</v>
+        <v>0.6418</v>
       </c>
       <c r="E214" t="n">
         <v>3</v>
@@ -6432,12 +6432,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6497,7 +6497,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>2.761</v>
+        <v>2.7609</v>
       </c>
       <c r="E217" t="n">
         <v>3</v>
@@ -6516,16 +6516,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>0.8598</v>
+        <v>0.8596</v>
       </c>
       <c r="E218" t="n">
         <v>1</v>
@@ -6544,12 +6544,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -6572,16 +6572,16 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>1.1472</v>
+        <v>1.1473</v>
       </c>
       <c r="E220" t="n">
         <v>3</v>
@@ -6600,16 +6600,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>0.5557</v>
+        <v>0.8176</v>
       </c>
       <c r="E221" t="n">
         <v>1</v>
@@ -6628,16 +6628,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>161390</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>0.6768999999999999</v>
+        <v>0.8375</v>
       </c>
       <c r="E222" t="n">
         <v>2</v>
@@ -6656,16 +6656,16 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>0.8176</v>
+        <v>0.9163</v>
       </c>
       <c r="E223" t="n">
         <v>3</v>
@@ -6684,16 +6684,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>0.3494</v>
+        <v>0.3492</v>
       </c>
       <c r="E224" t="n">
         <v>1</v>
@@ -6721,7 +6721,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>1.7099</v>
+        <v>1.71</v>
       </c>
       <c r="E225" t="n">
         <v>2</v>
@@ -6740,12 +6740,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6768,12 +6768,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>071050</t>
+          <t>011070</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>2.1558</v>
+        <v>2.1559</v>
       </c>
       <c r="E228" t="n">
         <v>2</v>
@@ -6824,16 +6824,16 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>2.2376</v>
+        <v>2.2375</v>
       </c>
       <c r="E229" t="n">
         <v>3</v>
@@ -6852,16 +6852,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0.538</v>
+        <v>1.043</v>
       </c>
       <c r="E230" t="n">
         <v>1</v>
@@ -6880,16 +6880,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>329180</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>1.043</v>
+        <v>1.4623</v>
       </c>
       <c r="E231" t="n">
         <v>2</v>
@@ -6908,23 +6908,23 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>003550</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>1.4623</v>
+        <v>10.6397</v>
       </c>
       <c r="E232" t="n">
         <v>3</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -6936,16 +6936,16 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>0.724</v>
+        <v>0.8277</v>
       </c>
       <c r="E233" t="n">
         <v>1</v>
@@ -6964,16 +6964,16 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>0.8282</v>
+        <v>1.04</v>
       </c>
       <c r="E234" t="n">
         <v>2</v>
@@ -6992,16 +6992,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>161390</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>0.9108000000000001</v>
+        <v>1.0702</v>
       </c>
       <c r="E235" t="n">
         <v>3</v>
@@ -7020,16 +7020,16 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>1.0415</v>
+        <v>1.2017</v>
       </c>
       <c r="E236" t="n">
         <v>1</v>
@@ -7048,16 +7048,16 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>267260</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>1.2008</v>
+        <v>1.2194</v>
       </c>
       <c r="E237" t="n">
         <v>2</v>
@@ -7076,16 +7076,16 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>1.222</v>
+        <v>1.4028</v>
       </c>
       <c r="E238" t="n">
         <v>3</v>
@@ -7132,12 +7132,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -7160,12 +7160,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -7197,7 +7197,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>6.5661</v>
+        <v>9.424899999999999</v>
       </c>
       <c r="E242" t="n">
         <v>1</v>
@@ -7216,16 +7216,16 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>6.6411</v>
+        <v>9.4772</v>
       </c>
       <c r="E243" t="n">
         <v>2</v>
@@ -7244,16 +7244,16 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>6.7117</v>
+        <v>9.5268</v>
       </c>
       <c r="E244" t="n">
         <v>3</v>
@@ -7272,16 +7272,16 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>0.8632</v>
+        <v>1.1829</v>
       </c>
       <c r="E245" t="n">
         <v>1</v>
@@ -7300,16 +7300,16 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>1.1849</v>
+        <v>1.2536</v>
       </c>
       <c r="E246" t="n">
         <v>2</v>
@@ -7328,16 +7328,16 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>028260</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>1.2168</v>
+        <v>1.3126</v>
       </c>
       <c r="E247" t="n">
         <v>3</v>
@@ -7356,16 +7356,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>086790</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>0.6803</v>
+        <v>0.9626</v>
       </c>
       <c r="E248" t="n">
         <v>1</v>
@@ -7384,16 +7384,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>010120</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>LS ELECTRIC</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>0.9631999999999999</v>
+        <v>0.9663</v>
       </c>
       <c r="E249" t="n">
         <v>2</v>
@@ -7412,16 +7412,16 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>0.9663</v>
+        <v>1.1165</v>
       </c>
       <c r="E250" t="n">
         <v>3</v>
@@ -7440,23 +7440,23 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>015760</t>
+          <t>030200</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>한국전력</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>1.3674</v>
+        <v>1.526</v>
       </c>
       <c r="E251" t="n">
         <v>1</v>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -7468,23 +7468,23 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>042660</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>1.4874</v>
+        <v>1.5765</v>
       </c>
       <c r="E252" t="n">
         <v>2</v>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -7496,16 +7496,16 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>064400</t>
+          <t>010120</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>LG씨엔에스</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>1.5261</v>
+        <v>1.6973</v>
       </c>
       <c r="E253" t="n">
         <v>3</v>
@@ -7524,16 +7524,16 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>161390</t>
+          <t>034020</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>0.3924</v>
+        <v>0.6036</v>
       </c>
       <c r="E254" t="n">
         <v>1</v>
@@ -7552,16 +7552,16 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>012330</t>
+          <t>267250</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>현대모비스</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>0.6038</v>
+        <v>0.6326000000000001</v>
       </c>
       <c r="E255" t="n">
         <v>2</v>
@@ -7580,16 +7580,16 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>005830</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>0.6322</v>
+        <v>0.6765</v>
       </c>
       <c r="E256" t="n">
         <v>3</v>
@@ -7617,7 +7617,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>0.5989</v>
+        <v>0.5991</v>
       </c>
       <c r="E257" t="n">
         <v>1</v>
@@ -7636,16 +7636,16 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>0.9495</v>
+        <v>0.9494</v>
       </c>
       <c r="E258" t="n">
         <v>2</v>
@@ -7664,12 +7664,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -7692,16 +7692,16 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>138040</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>0.8242</v>
+        <v>0.8226</v>
       </c>
       <c r="E260" t="n">
         <v>1</v>
@@ -7729,7 +7729,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>1.423</v>
+        <v>1.4225</v>
       </c>
       <c r="E261" t="n">
         <v>2</v>
@@ -7748,16 +7748,16 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>005387</t>
+          <t>086280</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>현대차2우B</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>1.7811</v>
+        <v>1.7804</v>
       </c>
       <c r="E262" t="n">
         <v>3</v>
@@ -7776,23 +7776,23 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>017670</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>1.1871</v>
+        <v>1.5578</v>
       </c>
       <c r="E263" t="n">
         <v>1</v>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>⚠</t>
         </is>
       </c>
     </row>
@@ -7804,16 +7804,16 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>1.5578</v>
+        <v>1.5605</v>
       </c>
       <c r="E264" t="n">
         <v>2</v>
@@ -7832,16 +7832,16 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>011200</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>1.5605</v>
+        <v>1.5926</v>
       </c>
       <c r="E265" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Add Rank 1 Only sheet to results.xlsx for portfolio construction
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Korean Stock → ARK Matches" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rank 1 Only" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15563,4 +15564,2338 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F89"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kr_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kr_company</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ark_sym</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>distance</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>flag</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>matched_by_n_ark_stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GRMN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.451</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TDY</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.501</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ITRN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.6675</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ALLT</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1.0357</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1.0474</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AUDC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1.1064</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1.2797</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RDWR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1.3467</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.3541</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CLBT</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1.3886</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1.5243</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NVMI</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1.5289</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CHKP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1.5703</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MNDY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1.7399</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1.7772</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1.8893</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>NYAX.TA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2.0227</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AVNT</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5991</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2.2491</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TBLA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>9.095599999999999</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>9.122400000000001</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>9.2135</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>9.2212</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>IRDM</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>9.3565</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RDCM</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>9.3758</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FVRR</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>9.412699999999999</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>9.418799999999999</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PINS</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>9.424899999999999</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>10.6747</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>270</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>VCYT</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.6326000000000001</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>270</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.6764</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>270</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>270</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ALGN</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>270</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>INMD</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1.3005</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>270</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CGEN</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1.6782</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>270</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2.8481</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1.2629</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2.8905</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ETOR</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>3.2116</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3.6827</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>4.2058</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>4.231</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>660</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1.4227</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>660</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2.1813</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>660</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>2.3541</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>660</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>4.7091</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>660</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>5.2391</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>12450</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>DDD</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.5424</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>12450</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>GILT</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.7701</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>12450</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PGY</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.8596</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>12450</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>TOST</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>0.8925</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>12450</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>7.9245</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>17670</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TATT</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0.4576</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>17670</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.5927</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>17670</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>LECO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>17670</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>PRLB</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1.1521</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>17670</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1.5578</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>68270</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BWXT</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0.5996</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>68270</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>1.2017</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>68270</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1.4153</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>68270</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>LHX</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>5.7889</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>267250</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HD현대</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>AME</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.8277</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>267250</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HD현대</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>HEI</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>1.0611</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>267250</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>HD현대</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CRS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>1.1829</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>267250</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HD현대</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ESLT.TA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1.6346</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>402340</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TSEM</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>402340</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CAMT</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1.3319</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>402340</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>3.1393</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>402340</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>6.1995</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>5490</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>POSCO홀딩스</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>KALU</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0.3492</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>5490</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>POSCO홀딩스</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>MTRN</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0.8226</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>5490</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>POSCO홀딩스</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>9.666399999999999</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>9540</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HD한국조선해양</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>MELI</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>0.6906</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>9540</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>HD한국조선해양</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0.8621</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>86790</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>LMT</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0.7204</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>86790</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ATI</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>0.9626</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>150</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>두산</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>KMDA.TA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>0.658</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>5930</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>삼성전자</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>2.1302</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>6800</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>미래에셋증권</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>11200</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>0.5203</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>15760</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>한국전력</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>3.1858</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>30200</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>JBL</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>1.526</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>32830</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>KTOS</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>1.0357</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>34020</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>두산에너빌리티</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>KMT</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0.6036</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>34730</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CCO.TO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>2.5743</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>64350</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>현대로템</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>MOG-A</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>0.6227</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>316140</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>우리금융지주</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>DKNG</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>2.5223</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>329180</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HD현대중공업</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>3.8892</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Portfolio (Rank1 < 1.5) sheet with deduplicated high-conviction Korean stocks
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Korean Stock → ARK Matches" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rank 1 Only" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio (Rank1 &lt; 1.5)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17898,4 +17899,506 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kr_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kr_company</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ark_stocks</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_ark_stocks</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>avg_distance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>min_distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>11070</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ALLT, AUDC, CLBT, CRM, GRMN, ITRN, RDWR, SHOP, TDY, TRMB</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.0178</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.451</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>270</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ALGN, ILMN, INMD, ISRG, VCYT</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9028</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.6326000000000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>17670</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>HON, LECO, PRLB, TATT</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.4576</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>12450</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DDD, GILT, PGY, TOST</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.7662</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.5424</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>267250</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HD현대</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AME, CRS, HEI</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.0239</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.8277</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>68270</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BWXT, CAT, GE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.0722</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.5996</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5490</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>POSCO홀딩스</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KALU, MTRN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5859</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.3492</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9540</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HD한국조선해양</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DASH, MELI</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.7764</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.6906</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>86790</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ATI, LMT</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.8415</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7204</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>402340</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CAMT, TSEM</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.211</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11200</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.5203</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.5203</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9150</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>삼성전기</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AVNT</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.5991</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.5991</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>34020</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>두산에너빌리티</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KMT</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.6036</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.6036</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>64350</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>현대로템</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MOG-A</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.6227</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.6227</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>150</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>두산</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KMDA.TA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.658</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.658</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>6800</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>미래에셋증권</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.9829</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>32830</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KTOS</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.0357</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.0357</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>307950</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>현대오토에버</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.2629</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.2629</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>660</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.4227</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.4227</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>